<commit_message>
Levellogik und target color balance, Flackern LEDs, MVC 2x, ongoing work on target color counterbalance
</commit_message>
<xml_diff>
--- a/experiments/experiment-1/levelBalance.xlsx
+++ b/experiments/experiment-1/levelBalance.xlsx
@@ -5,10 +5,10 @@
   <workbookPr defaultThemeVersion="166925"/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PhD-s\Apparatus\psychopy-apparatus-main\experiments\experiment-1\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\PhD-s\Repositories\psychopy-apparatus\psychopy-apparatus\experiments\experiment-1\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{EE89BCF8-A251-4734-9936-4A19958B81A6}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B26696DA-A432-4AB9-B050-6A7739413475}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-90" yWindow="-90" windowWidth="19380" windowHeight="11460" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -91,12 +91,220 @@
         </r>
       </text>
     </comment>
+    <comment ref="C2" authorId="0" shapeId="0" xr:uid="{3FF54933-61E0-433C-99CC-3C460DF37066}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A3" authorId="0" shapeId="0" xr:uid="{66605233-0004-4278-A47F-A62116D6CB0F}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="A4" authorId="0" shapeId="0" xr:uid="{9502CA91-7FB4-4BA0-9D12-0437E3992397}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C5" authorId="0" shapeId="0" xr:uid="{83ED8ADA-483E-40FB-BE8F-E498916A55DA}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C8" authorId="0" shapeId="0" xr:uid="{4CFE301C-F092-4E7D-8DAF-7D73339C5468}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C11" authorId="0" shapeId="0" xr:uid="{AA9336B0-3207-4855-BD3B-2DD124320589}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C14" authorId="0" shapeId="0" xr:uid="{3482CE0D-0502-4BA7-9C80-A5AAD467AF8E}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
+    <comment ref="C17" authorId="0" shapeId="0" xr:uid="{B851FEDD-6C57-431F-8F71-340D67663F36}">
+      <text>
+        <r>
+          <rPr>
+            <b/>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t xml:space="preserve">Values
+</t>
+        </r>
+        <r>
+          <rPr>
+            <sz val="10"/>
+            <color indexed="81"/>
+            <rFont val="Calibri Light"/>
+            <family val="2"/>
+            <scheme val="major"/>
+          </rPr>
+          <t>Each iteration of this loop, a different one of these values will be chosen. This will be the value of the variable named above.</t>
+        </r>
+      </text>
+    </comment>
   </commentList>
 </comments>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="8" uniqueCount="8">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="39" uniqueCount="12">
   <si>
     <t>deltaE</t>
   </si>
@@ -121,12 +329,24 @@
   <si>
     <t>0.28</t>
   </si>
+  <si>
+    <t>targetColor</t>
+  </si>
+  <si>
+    <t>0,0,255</t>
+  </si>
+  <si>
+    <t>255,0,0</t>
+  </si>
+  <si>
+    <t>0,255,0</t>
+  </si>
 </sst>
 </file>
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <styleSheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:x16r2="http://schemas.microsoft.com/office/spreadsheetml/2015/02/main" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" mc:Ignorable="x14ac x16r2 xr">
-  <fonts count="4" x14ac:knownFonts="1">
+  <fonts count="5" x14ac:knownFonts="1">
     <font>
       <sz val="11"/>
       <color theme="1"/>
@@ -156,6 +376,12 @@
       <name val="Calibri Light"/>
       <family val="2"/>
       <scheme val="major"/>
+    </font>
+    <font>
+      <sz val="8"/>
+      <name val="Calibri"/>
+      <family val="2"/>
+      <scheme val="minor"/>
     </font>
   </fonts>
   <fills count="3">
@@ -513,69 +739,223 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:xdr="http://schemas.openxmlformats.org/drawingml/2006/spreadsheetDrawing" xmlns:x14="http://schemas.microsoft.com/office/spreadsheetml/2009/9/main" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:B7"/>
+  <dimension ref="A1:C19"/>
   <sheetFormatPr baseColWidth="10" defaultColWidth="20.7265625" defaultRowHeight="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75"/>
   <cols>
     <col min="1" max="1" width="20.7265625" style="1"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:2" s="2" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+    <row r="1" spans="1:3" s="2" customFormat="1" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A1" s="2" t="s">
         <v>0</v>
       </c>
       <c r="B1" s="2" t="s">
         <v>1</v>
       </c>
-    </row>
-    <row r="2" spans="1:2" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="C1" s="2" t="s">
+        <v>8</v>
+      </c>
+    </row>
+    <row r="2" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A2" s="1">
         <v>10</v>
       </c>
       <c r="B2" t="s">
         <v>2</v>
       </c>
-    </row>
-    <row r="3" spans="1:2" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="C2" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="3" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
       <c r="A3" s="1">
+        <v>10</v>
+      </c>
+      <c r="B3" t="s">
+        <v>2</v>
+      </c>
+      <c r="C3" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="4" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A4" s="1">
+        <v>10</v>
+      </c>
+      <c r="B4" t="s">
+        <v>2</v>
+      </c>
+      <c r="C4" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="5" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A5" s="1">
         <v>20</v>
       </c>
-      <c r="B3" t="s">
+      <c r="B5" t="s">
         <v>5</v>
       </c>
-    </row>
-    <row r="4" spans="1:2" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A4" s="1">
+      <c r="C5" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="6" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A6" s="1">
+        <v>20</v>
+      </c>
+      <c r="B6" t="s">
+        <v>5</v>
+      </c>
+      <c r="C6" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="7" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A7" s="1">
+        <v>20</v>
+      </c>
+      <c r="B7" t="s">
+        <v>5</v>
+      </c>
+      <c r="C7" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="8" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A8" s="1">
         <v>30</v>
       </c>
-      <c r="B4" t="s">
+      <c r="B8" t="s">
         <v>6</v>
       </c>
-    </row>
-    <row r="5" spans="1:2" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A5" s="1">
+      <c r="C8" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="9" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A9" s="1">
+        <v>30</v>
+      </c>
+      <c r="B9" t="s">
+        <v>6</v>
+      </c>
+      <c r="C9" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="10" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A10" s="1">
+        <v>30</v>
+      </c>
+      <c r="B10" t="s">
+        <v>6</v>
+      </c>
+      <c r="C10" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="11" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A11" s="1">
         <v>40</v>
       </c>
-      <c r="B5" t="s">
+      <c r="B11" t="s">
         <v>7</v>
       </c>
-    </row>
-    <row r="6" spans="1:2" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A6" s="1">
+      <c r="C11" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="12" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A12" s="1">
+        <v>40</v>
+      </c>
+      <c r="B12" t="s">
+        <v>7</v>
+      </c>
+      <c r="C12" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="13" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A13" s="1">
+        <v>40</v>
+      </c>
+      <c r="B13" t="s">
+        <v>7</v>
+      </c>
+      <c r="C13" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="14" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A14" s="1">
         <v>50</v>
       </c>
-      <c r="B6" t="s">
+      <c r="B14" t="s">
         <v>4</v>
       </c>
-    </row>
-    <row r="7" spans="1:2" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
-      <c r="A7" s="1">
+      <c r="C14" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="15" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A15" s="1">
+        <v>50</v>
+      </c>
+      <c r="B15" t="s">
+        <v>4</v>
+      </c>
+      <c r="C15" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="16" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A16" s="1">
+        <v>50</v>
+      </c>
+      <c r="B16" t="s">
+        <v>4</v>
+      </c>
+      <c r="C16" s="1" t="s">
+        <v>11</v>
+      </c>
+    </row>
+    <row r="17" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A17" s="1">
         <v>60</v>
       </c>
-      <c r="B7" t="s">
+      <c r="B17" t="s">
         <v>3</v>
       </c>
+      <c r="C17" s="1" t="s">
+        <v>9</v>
+      </c>
+    </row>
+    <row r="18" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A18" s="1">
+        <v>60</v>
+      </c>
+      <c r="B18" t="s">
+        <v>3</v>
+      </c>
+      <c r="C18" s="1" t="s">
+        <v>10</v>
+      </c>
+    </row>
+    <row r="19" spans="1:3" ht="20.149999999999999" customHeight="1" x14ac:dyDescent="0.75">
+      <c r="A19" s="1">
+        <v>60</v>
+      </c>
+      <c r="B19" t="s">
+        <v>3</v>
+      </c>
+      <c r="C19" s="1" t="s">
+        <v>11</v>
+      </c>
     </row>
   </sheetData>
+  <phoneticPr fontId="4" type="noConversion"/>
   <dataValidations count="1">
     <dataValidation type="custom" allowBlank="1" showInputMessage="1" showErrorMessage="1" errorTitle="Invalid variable name" error="Variable names need to start with a letter or an underscore (_), followed by only letters, numbers and underscores." sqref="A1:XFD1" xr:uid="{7CD88A1A-7D71-4B66-8FF3-B42FC0AD4334}">
       <formula1>AND(ISNUMBER(SUMPRODUCT(SEARCH(MID(A1,ROW(INDIRECT("1:"&amp;LEN(A1))),1),"0123456789abcdefghijklmnopqrstuvwxyzABCDEFGHIJKLMNOPQRSTUVWXYZ_"))),ISNUMBER(SEARCH(LEFT(A1,1),"abcdefghijklmnopqrstuvwxyzABCDEFGHIJKLMNOPQRSTUVWXYZ_")),NOT(ISNUMBER(SEARCH("~*",A1))))</formula1>
@@ -588,6 +968,12 @@
 </file>
 
 <file path=customXml/item1.xml><?xml version="1.0" encoding="utf-8"?>
+<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
+  <documentManagement/>
+</p:properties>
+</file>
+
+<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
 <ct:contentTypeSchema xmlns:ct="http://schemas.microsoft.com/office/2006/metadata/contentType" xmlns:ma="http://schemas.microsoft.com/office/2006/metadata/properties/metaAttributes" ct:_="" ma:_="" ma:contentTypeName="Document" ma:contentTypeID="0x010100B9F5CAB0486A994CA2C3B13E059EF2AE" ma:contentTypeVersion="0" ma:contentTypeDescription="Een nieuw document maken." ma:contentTypeScope="" ma:versionID="8645ec4a60d0c8c7009d2d6675847a91">
   <xsd:schema xmlns:xsd="http://www.w3.org/2001/XMLSchema" xmlns:xs="http://www.w3.org/2001/XMLSchema" xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" targetNamespace="http://schemas.microsoft.com/office/2006/metadata/properties" ma:root="true" ma:fieldsID="636d7205651659ec4fcda0bcbde9384b">
     <xsd:element name="properties">
@@ -701,12 +1087,6 @@
 </ct:contentTypeSchema>
 </file>
 
-<file path=customXml/item2.xml><?xml version="1.0" encoding="utf-8"?>
-<p:properties xmlns:p="http://schemas.microsoft.com/office/2006/metadata/properties" xmlns:xsi="http://www.w3.org/2001/XMLSchema-instance" xmlns:pc="http://schemas.microsoft.com/office/infopath/2007/PartnerControls">
-  <documentManagement/>
-</p:properties>
-</file>
-
 <file path=customXml/item3.xml><?xml version="1.0" encoding="utf-8"?>
 <?mso-contentType ?>
 <FormTemplates xmlns="http://schemas.microsoft.com/sharepoint/v3/contenttype/forms">
@@ -717,6 +1097,21 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
+  <ds:schemaRefs>
+    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
+    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
+    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
+    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
+    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
+  </ds:schemaRefs>
+</ds:datastoreItem>
+</file>
+
+<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{EFF1C174-6AC6-4774-A736-3226A12360E4}">
   <ds:schemaRefs>
     <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/contentType"/>
@@ -732,21 +1127,6 @@
 </ds:datastoreItem>
 </file>
 
-<file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B3725960-8A89-4E70-9C40-340E0EDB6403}">
-  <ds:schemaRefs>
-    <ds:schemaRef ds:uri="http://purl.org/dc/elements/1.1/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/metadata/properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/dcmitype/"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/2006/documentManagement/types"/>
-    <ds:schemaRef ds:uri="http://www.w3.org/XML/1998/namespace"/>
-    <ds:schemaRef ds:uri="http://schemas.microsoft.com/office/infopath/2007/PartnerControls"/>
-    <ds:schemaRef ds:uri="http://schemas.openxmlformats.org/package/2006/metadata/core-properties"/>
-    <ds:schemaRef ds:uri="http://purl.org/dc/terms/"/>
-  </ds:schemaRefs>
-</ds:datastoreItem>
-</file>
-
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
 <ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{3744155D-8FAB-4E67-B5E0-C7FDBFB3715D}">
   <ds:schemaRefs>

</xml_diff>